<commit_message>
Day 5: PFMEA complete — data Occurrence, Action Priority, SC/CTQ, actions
- Injected data-driven Occurrence ratings into reports/PFMEA.xlsx from defect_rates.csv
- Implemented exact AIAG-VDA 2019 Action Priority (AP) calculation logic
- Identified 5 High-AP, 1 Medium-AP, and 3 Low-AP failure modes
- Finalized Critical Characteristic (CC ∇) and Significant Characteristic (SC) flags
- Formulated concrete Recommended Actions for all High-AP and Medium-AP risks
- Validated all 9 rows against AIAG-VDA standard assertions
</commit_message>
<xml_diff>
--- a/reports/PFMEA.xlsx
+++ b/reports/PFMEA.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -59,9 +59,9 @@
     </font>
     <font>
       <name val="Calibri"/>
-      <i val="1"/>
-      <color rgb="007030A0"/>
-      <sz val="9"/>
+      <b val="1"/>
+      <color rgb="00385723"/>
+      <sz val="9.5"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -69,8 +69,14 @@
       <color rgb="00C00000"/>
       <sz val="9.5"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00B25900"/>
+      <sz val="9.5"/>
+    </font>
   </fonts>
-  <fills count="13">
+  <fills count="16">
     <fill>
       <patternFill/>
     </fill>
@@ -127,8 +133,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00333f48"/>
-        <bgColor rgb="00333f48"/>
+        <fgColor rgb="00333F48"/>
+        <bgColor rgb="00333F48"/>
       </patternFill>
     </fill>
     <fill>
@@ -139,8 +145,26 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+        <bgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00FFFFFF"/>
         <bgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
+        <bgColor rgb="00FCE4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+        <bgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -184,7 +208,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -222,22 +246,25 @@
     <xf numFmtId="0" fontId="6" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="12" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="12" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="12" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="12" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="12" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="13" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="13" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="13" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="14" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="15" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="13" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -623,7 +650,7 @@
     <col width="10" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="32" customWidth="1" min="13" max="13"/>
+    <col width="34" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -704,7 +731,7 @@
       <c r="B4" s="3" t="n"/>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>M2 — Synchronized Risk Flowdown (Pass 1)</t>
+          <t>M2 — Final PFMEA with Data-Driven Occurrence</t>
         </is>
       </c>
       <c r="D4" s="3" t="n"/>
@@ -718,7 +745,7 @@
       <c r="H4" s="3" t="n"/>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t>2026-08-17 / Rev 1.0 (Draft)</t>
+          <t>2026-08-17 / Rev 2.0 (Complete)</t>
         </is>
       </c>
       <c r="J4" s="3" t="n"/>
@@ -805,7 +832,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="54" customHeight="1">
+    <row r="7" ht="56" customHeight="1">
       <c r="A7" s="12" t="inlineStr">
         <is>
           <t>OP10</t>
@@ -854,23 +881,21 @@
       <c r="J7" s="12" t="n">
         <v>6</v>
       </c>
-      <c r="K7" s="15" t="inlineStr">
-        <is>
-          <t>TBD-D5</t>
-        </is>
+      <c r="K7" s="12" t="n">
+        <v>1</v>
       </c>
       <c r="L7" s="15" t="inlineStr">
         <is>
-          <t>TBD-D5</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="M7" s="13" t="inlineStr">
         <is>
-          <t>Maintain current PM schedule; verify weighing record in Control Plan OP10.</t>
+          <t>Current PM schedule and periodic scale checks are adequate (Low AP, O=1). Maintain standard work instructions.</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="54" customHeight="1">
+    <row r="8" ht="56" customHeight="1">
       <c r="A8" s="16" t="inlineStr">
         <is>
           <t>OP20</t>
@@ -919,23 +944,21 @@
       <c r="J8" s="16" t="n">
         <v>6</v>
       </c>
-      <c r="K8" s="19" t="inlineStr">
-        <is>
-          <t>TBD-D5</t>
-        </is>
+      <c r="K8" s="16" t="n">
+        <v>10</v>
       </c>
       <c r="L8" s="19" t="inlineStr">
         <is>
-          <t>TBD-D5</t>
+          <t>High</t>
         </is>
       </c>
       <c r="M8" s="17" t="inlineStr">
         <is>
-          <t>Flagged as Significant Characteristic (SC); establish dedicated optical/stylus measurement and reaction rule.</t>
+          <t>HIGH AP (O=10, 22.3%): Implement automated spindle vibration monitoring + optical non-contact profilometer inspection (5 parts/shift); index inserts at 150 parts.</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="54" customHeight="1">
+    <row r="9" ht="56" customHeight="1">
       <c r="A9" s="12" t="inlineStr">
         <is>
           <t>OP20</t>
@@ -984,23 +1007,21 @@
       <c r="J9" s="12" t="n">
         <v>6</v>
       </c>
-      <c r="K9" s="15" t="inlineStr">
-        <is>
-          <t>TBD-D5</t>
-        </is>
-      </c>
-      <c r="L9" s="15" t="inlineStr">
-        <is>
-          <t>TBD-D5</t>
+      <c r="K9" s="12" t="n">
+        <v>9</v>
+      </c>
+      <c r="L9" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="M9" s="13" t="inlineStr">
         <is>
-          <t>Add fixture cleaning verification to daily operator autonomous maintenance checklist.</t>
+          <t>HIGH AP (O=9, 8.4%): Install automated pneumatic seating interlock with CNC start block; add fixture chip inspection to daily operator checklist.</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="54" customHeight="1">
+    <row r="10" ht="56" customHeight="1">
       <c r="A10" s="16" t="inlineStr">
         <is>
           <t>OP20</t>
@@ -1049,23 +1070,21 @@
       <c r="J10" s="16" t="n">
         <v>6</v>
       </c>
-      <c r="K10" s="19" t="inlineStr">
-        <is>
-          <t>TBD-D5</t>
-        </is>
-      </c>
-      <c r="L10" s="19" t="inlineStr">
-        <is>
-          <t>TBD-D5</t>
+      <c r="K10" s="16" t="n">
+        <v>7</v>
+      </c>
+      <c r="L10" s="20" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
       <c r="M10" s="17" t="inlineStr">
         <is>
-          <t>Designate as SC; flow down to Control Plan with calibrated depth micrometer inspection.</t>
+          <t>MEDIUM AP (O=7, 1.4%): Flow down SC to Control Plan; mandate digital depth micrometer with wireless SPC data capture (2 parts/shift).</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="54" customHeight="1">
+    <row r="11" ht="56" customHeight="1">
       <c r="A11" s="12" t="inlineStr">
         <is>
           <t>OP20</t>
@@ -1114,23 +1133,21 @@
       <c r="J11" s="12" t="n">
         <v>5</v>
       </c>
-      <c r="K11" s="15" t="inlineStr">
-        <is>
-          <t>TBD-D5</t>
-        </is>
-      </c>
-      <c r="L11" s="15" t="inlineStr">
-        <is>
-          <t>TBD-D5</t>
+      <c r="K11" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="L11" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="M11" s="13" t="inlineStr">
         <is>
-          <t>Include Go/No-Go plug gauge calibration in gauge repeatability and reproducibility (GR&amp;R) schedule.</t>
+          <t>HIGH AP (O=8, 2.4%): Replace manual plug gauge with calibrated three-point internal bore micrometer; quarterly CNC dynamic circularity calibration.</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="54" customHeight="1">
+    <row r="12" ht="56" customHeight="1">
       <c r="A12" s="16" t="inlineStr">
         <is>
           <t>OP30</t>
@@ -1179,23 +1196,21 @@
       <c r="J12" s="16" t="n">
         <v>5</v>
       </c>
-      <c r="K12" s="19" t="inlineStr">
-        <is>
-          <t>TBD-D5</t>
-        </is>
+      <c r="K12" s="16" t="n">
+        <v>10</v>
       </c>
       <c r="L12" s="19" t="inlineStr">
         <is>
-          <t>TBD-D5</t>
+          <t>High</t>
         </is>
       </c>
       <c r="M12" s="17" t="inlineStr">
         <is>
-          <t>CRITICAL CHARACTERISTIC (∇): Mandatory Control Plan flowdown; evaluate 100% automated runout gauging.</t>
+          <t>HIGH AP &amp; CRITICAL CHARACTERISTIC (∇) (O=10, 12.9%): Integrate 100% automated in-line laser runout gauge on lathe unloader arm with auto-reject gate.</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="54" customHeight="1">
+    <row r="13" ht="56" customHeight="1">
       <c r="A13" s="12" t="inlineStr">
         <is>
           <t>OP30</t>
@@ -1244,23 +1259,21 @@
       <c r="J13" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="K13" s="15" t="inlineStr">
-        <is>
-          <t>TBD-D5</t>
-        </is>
+      <c r="K13" s="12" t="n">
+        <v>7</v>
       </c>
       <c r="L13" s="15" t="inlineStr">
         <is>
-          <t>TBD-D5</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="M13" s="13" t="inlineStr">
         <is>
-          <t>Implement SPC variable chart on piston rod OD in Control Plan OP30.</t>
+          <t>Low AP (O=7, D=4). Maintain touch-probe tool compensation and X-bar/R control chart at station in Control Plan.</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="54" customHeight="1">
+    <row r="14" ht="56" customHeight="1">
       <c r="A14" s="16" t="inlineStr">
         <is>
           <t>OP30</t>
@@ -1286,7 +1299,7 @@
       <c r="E14" s="16" t="n">
         <v>6</v>
       </c>
-      <c r="F14" s="20" t="inlineStr">
+      <c r="F14" s="21" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1309,23 +1322,21 @@
       <c r="J14" s="16" t="n">
         <v>5</v>
       </c>
-      <c r="K14" s="19" t="inlineStr">
-        <is>
-          <t>TBD-D5</t>
-        </is>
-      </c>
-      <c r="L14" s="19" t="inlineStr">
-        <is>
-          <t>TBD-D5</t>
+      <c r="K14" s="16" t="n">
+        <v>6</v>
+      </c>
+      <c r="L14" s="15" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
       <c r="M14" s="17" t="inlineStr">
         <is>
-          <t>Verify Z-axis datum touch-off procedure in standard work instruction.</t>
+          <t>Low AP (O=6, 0.2%). Maintain positive chuck stop standard and hourly height gauge inspection.</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="54" customHeight="1">
+    <row r="15" ht="56" customHeight="1">
       <c r="A15" s="12" t="inlineStr">
         <is>
           <t>OP40</t>
@@ -1351,7 +1362,7 @@
       <c r="E15" s="12" t="n">
         <v>8</v>
       </c>
-      <c r="F15" s="21" t="inlineStr">
+      <c r="F15" s="22" t="inlineStr">
         <is>
           <t>SC</t>
         </is>
@@ -1374,19 +1385,17 @@
       <c r="J15" s="12" t="n">
         <v>3</v>
       </c>
-      <c r="K15" s="15" t="inlineStr">
-        <is>
-          <t>TBD-D5</t>
-        </is>
-      </c>
-      <c r="L15" s="15" t="inlineStr">
-        <is>
-          <t>TBD-D5</t>
+      <c r="K15" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="L15" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="M15" s="13" t="inlineStr">
         <is>
-          <t>100% automated in-line signature monitoring documented as primary detection control in Control Plan OP40.</t>
+          <t>HIGH AP (O=8, 2.4%): Maintain 100% automated force-displacement press signature analysis with automatic interlock; calibrate load cell weekly.</t>
         </is>
       </c>
     </row>

</xml_diff>